<commit_message>
feat(w15): OCR bảng điểm có confidence và kiểm chéo
- w15_ocr: vẽ bảng điểm tổng hợp (Mẫu In D5050A0), OCR Tesseract theo dải cột,
  kiểm chéo mã/TC/R-B02/tổng TC/ĐTBCHK, HP không chắc → solver xét F/D/A
- Kết quả: fact nhận đúng 783/784, 0/18 kết luận sai, độ phủ 1/18
- Sửa 2 lỗi soundness từ review (F/A không đơn điệu theo GPA; học lại)
- Schema: thêm ocr_raw, mô tả confidence; .gitignore dữ liệu bảng điểm thật
- Báo cáo Tuan15, cập nhật Excel và CLAUDE.md (bài học)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1748,10 +1748,14 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>09/10/2026: OCR pipeline v1 (w15_ocr/) — Tesseract vie + OCR theo dải cột có whitelist; kiểm chéo mã∈CTĐT, TC, R-B02, tổng TC học kỳ, ĐTBCHK; confidence + ocr_raw mỗi fact. Ảnh tổng hợp 6 hồ sơ × 3 nhiễu: fact nhận đúng 783/784 (0,999), 0/18 kết luận sai, độ phủ chỉ 1/18 (còn lại UNKNOWN). Bảng điểm thật (không commit): trang 1 nhận 10/11, đúng 10/10. Review tìm 2 lỗi soundness (F/A không đơn điệu theo GPA; học lại) — đã sửa, có test. Phát hiện: KB Tuần 10 thế giới đóng cho xac_nhan_ky_luat_sach (FALSE thay vì UNKNOWN) → Tuần 16; bảng điểm thật ghi CC004 (miễn AV) và GDTC TC025–027, KB chỉ có TC100 → cần xác minh.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2784,25 +2788,29 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Đọc: không có phần đọc tài liệu OCR mới | Code: render_transcript.py, ocr_transcript.py, validate_ocr.py | Test: A chuẩn hoá, B 18 ca tổng hợp, C 3 ca tiêm lỗi, E 2 ca hồi quy, D bảng điểm thật | Artifact: Tuan15_OCR_Bang_Diem.md | Lỗi/phát hiện: F/A không đơn điệu; học lại; thế giới đóng ở KB; CC004; GDTC TC025–027; xoay -0,05° làm hỏng OCR</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">

</xml_diff>

<commit_message>
feat(w16): abstention engine — ba trị, missing evidence, không đoán khi thiếu dữ liệu
- graduation_solver.lp mục 0: mở nhánh dữ kiện ngoài chưa khai báo
  (xac_nhan_ky_luat_sach, qua_thoi_gian_toi_da) thay giả định thế giới đóng (P15-2)
- loader w7/w11/w12: khai_bao(ky_luat) khi khai báo false; nạp da_hoc_nam2, tc_cong_nhan
- w16_abstention/abstention.py: chỉ hỏi dữ kiện quyết định, kèm câu hỏi, nguồn,
  kết luận theo từng giá trị; UNKNOWN → ket_luan None, không theo đa số
- prototype w12 dùng missing evidence mới; bỏ đường dẫn D:/
- w10 B6: thiếu xác nhận kỷ luật → UNKNOWN (trước: FALSE) + B6b khai báo false → FALSE
- 6 hồ sơ giả lập thêm da_hoc_nam2 = 9; w15 chuyển tiếp da_hoc_nam2/tc_cong_nhan
- Báo cáo Tuan16_Abstention_Engine.md, cập nhật kế hoạch Excel, bài học CLAUDE.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22188" windowHeight="9000" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Kế hoạch 24 tuần" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Checklist tuần" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tổng hợp giai đoạn" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kế hoạch 24 tuần" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist tuần" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng hợp giai đoạn" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Kế hoạch 24 tuần'!$A$1:$H$25</definedName>
@@ -1790,10 +1790,14 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>14/10/2026: Abstention engine v1 (w16_abstention/). KB mở nhánh dữ kiện ngoài chưa khai báo (xac_nhan_ky_luat_sach, qua_thoi_gian_toi_da) → UNKNOWN thay vì FALSE/"chưa quá hạn" (sửa P15-2); missing evidence = chỉ dữ kiện QUYẾT ĐỊNH + câu hỏi + nguồn + kết luận theo từng giá trị; UNKNOWN → không kết luận, không theo đa số. validate_abstention 28/28 (tự soạn; 14 fail với luật cũ), mọi tuần 5–16 ĐẠT. LƯU Ý: P16-2 tot_nghiep chưa phụ thuộc điều kiện thời gian (R-Formal Đ32 k1 vs Đ5) — cần quyết định diễn giải; tc_cong_nhan vẫn thế giới đóng.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2823,25 +2827,29 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Đọc: không có phần đọc tài liệu ba trị/abstention mới | Code: abstention.py, graduation_solver.lp mục 0, loader w7/w11/w12 | Test: validate_abstention 28/28 (A9 B10 C5 D4), w10 B6 đổi FALSE→UNKNOWN + B6b | Artifact: Tuan16_Abstention_Engine.md | Lỗi/phát hiện: khai_bao tự triệt nhánh (P16-1); tot_nghiep bỏ qua thời gian (P16-2, chưa sửa); tc_cong_nhan thế giới đóng; đường dẫn D:/ &amp; font Windows; g10 nhiều giá trị/mô hình</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">

</xml_diff>

<commit_message>
fix(rformal): tốt nghiệp phải trong thời gian tối đa (Điều 5) — P16-2
- R-Formal v1.7: tot_nghiep thêm `not qua_thoi_gian_toi_da` (QĐ3266 Đ5, tr.4:
  thời gian tối đa để SV hoàn thành CTĐT; CTĐT 4,5 năm → 9 năm)
- graduation_solver.lp: tot_nghiep thêm dk_thoi_gian (du_dk_hoc_vu còn được
  R-Formal định nghĩa không có thời gian nên đặt ở đó không chặn được)
- Hồi quy fail với luật cũ: w5 C9b, w10 B7b/B7d, w16 A10/A11; biên C9c, B7c
- Fixture KY_LUAT w10/w11 thêm da_hoc_nam2(9); cập nhật báo cáo, Excel, CLAUDE.md
- Học phí ×1,5 chưa hình thức hoá: không có trong QĐ3266/QĐ5339

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1795,7 +1795,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>14/10/2026: Abstention engine v1 (w16_abstention/). KB mở nhánh dữ kiện ngoài chưa khai báo (xac_nhan_ky_luat_sach, qua_thoi_gian_toi_da) → UNKNOWN thay vì FALSE/"chưa quá hạn" (sửa P15-2); missing evidence = chỉ dữ kiện QUYẾT ĐỊNH + câu hỏi + nguồn + kết luận theo từng giá trị; UNKNOWN → không kết luận, không theo đa số. validate_abstention 28/28 (tự soạn; 14 fail với luật cũ), mọi tuần 5–16 ĐẠT. LƯU Ý: P16-2 tot_nghiep chưa phụ thuộc điều kiện thời gian (R-Formal Đ32 k1 vs Đ5) — cần quyết định diễn giải; tc_cong_nhan vẫn thế giới đóng.</t>
+          <t>14/10/2026: Abstention engine v1 (w16_abstention/). KB mở nhánh dữ kiện ngoài chưa khai báo (xac_nhan_ky_luat_sach, qua_thoi_gian_toi_da) → UNKNOWN thay vì FALSE/"chưa quá hạn" (sửa P15-2); missing evidence = chỉ dữ kiện QUYẾT ĐỊNH + câu hỏi + nguồn + kết luận theo từng giá trị; UNKNOWN → không kết luận, không theo đa số. validate_abstention 30/30 (tự soạn; 14 fail với luật cũ), mọi tuần 5–16 ĐẠT. P16-2 đã sửa 17/10/2026 (chọn cách đọc b): quá thời gian tối đa (Đ5, CTĐT 4,5 năm → 9 năm) thì không tốt nghiệp — R-Formal v1.7 + graduation_solver, 5 ca hồi quy fail với luật cũ. LƯU Ý: tc_cong_nhan vẫn thế giới đóng; học phí ×1,5 sau thời gian thiết kế chưa có văn bản nguồn (không có trong QĐ3266/QĐ5339) → chưa hình thức hoá.</t>
         </is>
       </c>
     </row>
@@ -2847,7 +2847,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không có phần đọc tài liệu ba trị/abstention mới | Code: abstention.py, graduation_solver.lp mục 0, loader w7/w11/w12 | Test: validate_abstention 28/28 (A9 B10 C5 D4), w10 B6 đổi FALSE→UNKNOWN + B6b | Artifact: Tuan16_Abstention_Engine.md | Lỗi/phát hiện: khai_bao tự triệt nhánh (P16-1); tot_nghiep bỏ qua thời gian (P16-2, chưa sửa); tc_cong_nhan thế giới đóng; đường dẫn D:/ &amp; font Windows; g10 nhiều giá trị/mô hình</t>
+          <t>Đọc: không có phần đọc tài liệu ba trị/abstention mới | Code: abstention.py, graduation_solver.lp mục 0, loader w7/w11/w12 | Test: validate_abstention 30/30 (A11 B10 C5 D4); hồi quy P16-2 w5 C9b/c, w10 B7b–d, w10 B6 đổi FALSE→UNKNOWN + B6b | Artifact: Tuan16_Abstention_Engine.md | Lỗi/phát hiện: khai_bao tự triệt nhánh (P16-1); tot_nghiep bỏ qua thời gian (P16-2, đã sửa v1.7); tc_cong_nhan thế giới đóng; đường dẫn D:/ &amp; font Windows; g10 nhiều giá trị/mô hình</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(w17): chấm CPA² trên adversarial set + báo cáo Tuần 17
- run_adversarial.py: Soundness/Coverage/Selective Acc/từ chối thừa/hỏi đúng theo dev/test;
  bắt lỗi từng ca; ca khong_phat_hien_duoc báo riêng (errata E17-1)
- Kết quả test (37 ca): Soundness 91,9%, Coverage 78,4%, SelAcc 89,7%, từ chối thừa 0;
  ngoài nhóm hồ sơ lỗi không sai ca nào (72/72 dev+test)
- Phát hiện: P17-1 hồ sơ mâu thuẫn 0/6 sound; P17-2 lỗi OCR nhất quán 2/2;
  P17-3 Đ6 k1 3 HK/năm → R-Formal trừ trần thời gian sai đơn vị (chưa sửa)
- Review: nguồn thêm số trang; gold_dong_bang.json trích từ 200b860 + validate G1/G2
  chống sửa gold; dau_vao_baseline() không lộ đáp án; gold KHÔNG đổi
- Báo cáo Tuan17_Adversarial_Set.md, Excel dòng 17, CLAUDE.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1832,10 +1832,14 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>17/10/2026: Adversarial set v1 (w17_adversarial/) — 80 ca chấm điểm (thiếu dữ liệu 17, sát ngưỡng 24, bẫy quy chế 15, hồ sơ lỗi 6, OCR sai mức tài liệu 18) + 5 ca không chấm; gold viết tay kèm nguồn điều/khoản/trang, ĐÓNG BĂNG ở commit 200b860 trước khi chạy; oracle Python độc lập kiểm 29 tiền đề; dev/test phân tầng. CPA² test (37 ca): Soundness 91,9%, Coverage 78,4%, SelAcc 89,7%, từ chối thừa 0. LƯU Ý: hồ sơ mâu thuẫn 0/6 sound (P17-1, loader tin mọi bản ghi); lỗi OCR nhất quán 2/2 trái sự thật (P17-2); đơn vị HK trong trần thời gian sai (Đ6: 3 HK/năm, P17-3); gold tự soạn, chưa đo κ.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2862,25 +2866,29 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Đọc: không có phần đọc tài liệu adversarial evaluation mới (chỉ đọc lại QĐ3266/QĐ5339 để lấy nguồn gold) | Code: build_adversarial.py, oracle.py, dau_vao.py, run_adversarial.py, validate_adversarial.py | Test/Dataset: 80 ca (dev 41/test 39), gold đóng băng 200b860 | Artifact: adversarial_set.json + Tuan17_Adversarial_Set.md | Lỗi/phát hiện: P17-1 hồ sơ mâu thuẫn 0/6; P17-2 OCR nhất quán 2/2; P17-3 1 HK = 1/3 năm (Đ6 k1); errata E17-1…5</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">

</xml_diff>

<commit_message>
fix(w17): sửa P17-1/P17-2/P17-3 phát hiện từ bộ đối kháng
- P17-1: abstention.ra_soat() — bản ghi điểm tự mâu thuẫn (ngoài thang, chữ ≠ quy đổi
  Đ22 k2, trạng thái ≠ ngưỡng D, TC ≠ CTĐT, M/W/I kèm điểm) → bỏ, mở F/D/A (+ giá trị ghi);
  thời gian học không thể (> 20 TC/HK, Đ14 k1) → coi như chưa khai báo; gọi ở w16/w12/w11/w15
- P17-3: R-Formal v1.8 — trần thời gian theo HK (QĐ3266 Đ6 k1: 3 HK/năm),
  thoi_gian_toi_da_hk, so 3·da_hoc_nam2 > 2·M; hồi quy w5 C16b, w10 B7e fail với luật cũ
- P17-2: w15 — ĐTBCHK không đọc được → học kỳ không tin; mã bắt buộc đọc nhầm thành mã
  lệch 1 ký tự cùng TC → cả hai không chắc (w15 F1–F4)
- Chạy lại bộ đối kháng ra file *_sau_P17 (test đã nhiễm); số chính thức Tuần 17 giữ nguyên;
  gold không đổi (G2 khớp 200b860); errata E17-6
- Báo cáo Tuần 16/17, Excel dòng 17, CLAUDE.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1837,7 +1837,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>17/10/2026: Adversarial set v1 (w17_adversarial/) — 80 ca chấm điểm (thiếu dữ liệu 17, sát ngưỡng 24, bẫy quy chế 15, hồ sơ lỗi 6, OCR sai mức tài liệu 18) + 5 ca không chấm; gold viết tay kèm nguồn điều/khoản/trang, ĐÓNG BĂNG ở commit 200b860 trước khi chạy; oracle Python độc lập kiểm 29 tiền đề; dev/test phân tầng. CPA² test (37 ca): Soundness 91,9%, Coverage 78,4%, SelAcc 89,7%, từ chối thừa 0. LƯU Ý: hồ sơ mâu thuẫn 0/6 sound (P17-1, loader tin mọi bản ghi); lỗi OCR nhất quán 2/2 trái sự thật (P17-2); đơn vị HK trong trần thời gian sai (Đ6: 3 HK/năm, P17-3); gold tự soạn, chưa đo κ.</t>
+          <t>17/10/2026: Adversarial set v1 (w17_adversarial/) — 80 ca chấm điểm (thiếu dữ liệu 17, sát ngưỡng 24, bẫy quy chế 15, hồ sơ lỗi 6, OCR sai mức tài liệu 18) + 5 ca không chấm; gold viết tay kèm nguồn điều/khoản/trang, ĐÓNG BĂNG ở commit 200b860 trước khi chạy; oracle Python độc lập kiểm 29 tiền đề; dev/test phân tầng. CPA² test (37 ca): Soundness 91,9%, Coverage 78,4%, SelAcc 89,7%, từ chối thừa 0. SỬA 18/10/2026: P17-1 rà soát hồ sơ mâu thuẫn (abstention.ra_soat), P17-2 OCR (ĐTBCHK không đọc được; mã bắt buộc đọc nhầm), P17-3 R-Formal v1.8 trần theo HK (Đ6 k1: 3 HK/năm). Chạy lại: dev/test 100% sound, 0/2 rủi ro OCR ẩn — NHƯNG test đã nhiễm (sửa sau khi thấy ca test) → cần bộ test mới ở Tuần 20. LƯU Ý: số chính thức T17 giữ nguyên; gold tự soạn, chưa đo κ; 3 bản loader chưa gộp.</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không có phần đọc tài liệu adversarial evaluation mới (chỉ đọc lại QĐ3266/QĐ5339 để lấy nguồn gold) | Code: build_adversarial.py, oracle.py, dau_vao.py, run_adversarial.py, validate_adversarial.py | Test/Dataset: 80 ca (dev 41/test 39), gold đóng băng 200b860 | Artifact: adversarial_set.json + Tuan17_Adversarial_Set.md | Lỗi/phát hiện: P17-1 hồ sơ mâu thuẫn 0/6; P17-2 OCR nhất quán 2/2; P17-3 1 HK = 1/3 năm (Đ6 k1); errata E17-1…5</t>
+          <t>Đọc: không có phần đọc tài liệu adversarial evaluation mới (chỉ đọc lại QĐ3266/QĐ5339 để lấy nguồn gold) | Code: build_adversarial.py, oracle.py, dau_vao.py, run_adversarial.py, validate_adversarial.py | Test/Dataset: 80 ca (dev 41/test 39), gold đóng băng 200b860 | Artifact: adversarial_set.json + Tuan17_Adversarial_Set.md | Lỗi/phát hiện: P17-1 hồ sơ mâu thuẫn 0/6; P17-2 OCR nhất quán 2/2; P17-3 1 HK = 1/3 năm (Đ6 k1); errata E17-1…5 | Sau T17: sửa P17-1/2/3 (TDD: w16 E1–E12, w15 F1–F4, w5 C16b, w10 B7e)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(w18): eligibility engine — LVTN/TLTN/niên luận/thực tập/thay thế ba trị
- eligibility.lp/.py: ELIGIBLE / NOT_ELIGIBLE / UNKNOWN / DA_HOAN_THANH / MAU_THUAN,
  lý do (thieu_tc, thieu_tien_quyet, dv_cong_bo_khac), chứng chỉ điều/khoản, câu hỏi bổ sung
- QĐ3266 Đ31 (R-F04): điều kiện nhận đề tài do đơn vị đào tạo quy định → không bịa,
  nhận kết quả xét qua hinh_thuc_cuoi_khoa (schema + loader); thiếu → UNKNOWN
- R-F04 thêm rule_src r_f04 + asp trong catalog (vẫn lớp N); corpus sinh lại (1 passage)
- prototype: "đủ điều kiện làm luận văn/tiểu luận" đi qua eligibility — sửa P18-1
  (claim du_dk_tc không đối số → luôn FALSE); không hồ sơ → UNKNOWN; hậu kiểm mã HP
- validate_eligibility 36/36 (gold viết tay trước); L3 chặn thêm khai_bao(hinh_thuc)
- Báo cáo Tuan18_Eligibility.md, Excel dòng 18, CLAUDE.md, Viec_ton_dong A12

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1874,10 +1874,14 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>18/10/2026: Eligibility module v1 (w18_eligibility/) — ELIGIBLE/NOT_ELIGIBLE/UNKNOWN (+DA_HOAN_THANH, MAU_THUAN) cho LVTN, TLTN, niên luận, niên luận cơ sở, thực tập, tích lũy TC thay LVTN (Đ31 k3), HP thay thế (QĐ5339 Đ3 k9); lý do (thiếu TC/tiên quyết) + chứng chỉ điều/khoản + câu hỏi bổ sung. validate_eligibility 36/36 (tự soạn), mọi tuần 5–18 ĐẠT. Phát hiện P18-1: prototype luôn FALSE cho "đủ điều kiện làm luận văn" (claim du_dk_tc không đối số) — đã sửa. LƯU Ý: điều kiện nhận đề tài LVTN/TLTN do đơn vị đào tạo quy định (Đ31, R-F04) — chưa có văn bản → chỉ nhận kết quả xét (hinh_thuc_cuoi_khoa), thiếu → UNKNOWN.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2901,25 +2905,29 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Đọc: không có phần đọc tài liệu mới (chỉ đối chiếu QĐ3266 Đ31, CTĐT) | Code: eligibility.lp, eligibility.py, prototype.answer_eligibility, loader hinh_thuc_cuoi_khoa | Test: validate_eligibility 36/36 | Artifact: Tuan18_Eligibility.md | Lỗi/phát hiện: P18-1 claim du_dk_tc không đối số → luôn FALSE; P18-2 đủ TC ≠ đủ ĐK (R-F04); P18-3 đã xong hình thức khác</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">

</xml_diff>

<commit_message>
feat(w19): Recommendation v1 — chỉ đề xuất phương án đã chứng minh hợp lệ
- w19_recommendation: ứng viên ba trị (hợp lệ trên mọi thế giới) + clingo tối ưu
  ≤ 20 TC (R-C01), nhóm một nhánh, không dư nhóm; ưu tiên là chính sách tư vấn;
  UNKNOWN → can_xac_minh; hình thức tốt nghiệp qua Eligibility; xin miễn (QD-11);
  thay thế (R-M13); kiểm lại phương án tường minh
- QD-13: song hành học trước/cùng/sau (xác nhận ngoài văn bản) — KB giữ R-A04,
  chỉ là lời khuyên; catalog + phụ lục sinh lại
- prototype: ý định de_xuat, học kỳ trong câu hỏi, chuẩn hoá NFC
- validate_recommendation 34/34; mọi tuần 5–19 ĐẠT

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1916,10 +1916,14 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>18/10/2026: Recommendation v1 (w19_recommendation/) — đề xuất đăng ký 1 HK (hk 1/2/3): ứng viên hợp lệ trên MỌI thế giới (du_dk_dang_ky TRUE, chưa tích lũy, mở HK, cần cho CTĐT; nhóm một nhánh), clingo tối ưu ≤20 TC (R-C01) + ưu tiên CHÍNH SÁCH (bắt buộc → mở khóa → song hành → nhóm → TC); UNKNOWN → cần xác minh; hình thức tốt nghiệp qua Eligibility; xin miễn (nộp đơn, QD-11); thay thế (R-M13). validate_recommendation 34/34 (tự soạn), bất biến kiểm lại độc lập 21 lần đề xuất, mọi tuần 5–19 ĐẠT. QD-13 (Loi 18/10/2026): song hành học trước/cùng/sau — KHÁC câu chữ Đ7 k5 → KB giữ R-A04, chỉ là lời khuyên. Phát hiện P19-1 (đủ ĐK xin miễn ≠ cần), P19-2 (AV tăng cường trước căn bản), P19-3 (parser kì/kỳ, HK4, NFD). Hạn chế: chỉ 1 HK, chưa lịch học.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2940,25 +2944,29 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Đọc: không có phần đọc tài liệu mới | Code: recommendation.py, recommendation.lp, prototype.answer_recommendation + parser de_xuat | Test: validate_recommendation 34/34 | Artifact: Tuan19_Recommendation.md | Lỗi/phát hiện: P19-1 đủ ĐK xin miễn ≠ cần; P19-2 ưu tiên TC chọn AV tăng cường trước căn bản; P19-3 parser học kỳ/ý định</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">

</xml_diff>

<commit_message>
fix(w19): song hành theo đúng QĐ3266 Đ7 k5 — rút lại QD-13
- Đối chiếu PDF gốc: song hành "phải học trước hoặc học cùng lúc" → QD-13
  (học sau cũng được) rút lại; catalog R-A04 + phụ lục sinh lại
- Recommendation: ràng buộc cứng — HP song hành đã học (có bản ghi, kể cả F;
  W không tính) hoặc chọn cùng kỳ; không thoả → khong_du_song_hanh (Đ7 k5);
  chưa chắc → can_xac_minh; chứng chỉ song_hanh ← r_a04
- validate_recommendation 39/39 (F1, F3, F5, F6 fail trước khi sửa);
  mọi tuần 5–19 ĐẠT

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1921,7 +1921,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>18/10/2026: Recommendation v1 (w19_recommendation/) — đề xuất đăng ký 1 HK (hk 1/2/3): ứng viên hợp lệ trên MỌI thế giới (du_dk_dang_ky TRUE, chưa tích lũy, mở HK, cần cho CTĐT; nhóm một nhánh), clingo tối ưu ≤20 TC (R-C01) + ưu tiên CHÍNH SÁCH (bắt buộc → mở khóa → song hành → nhóm → TC); UNKNOWN → cần xác minh; hình thức tốt nghiệp qua Eligibility; xin miễn (nộp đơn, QD-11); thay thế (R-M13). validate_recommendation 34/34 (tự soạn), bất biến kiểm lại độc lập 21 lần đề xuất, mọi tuần 5–19 ĐẠT. QD-13 (Loi 18/10/2026): song hành học trước/cùng/sau — KHÁC câu chữ Đ7 k5 → KB giữ R-A04, chỉ là lời khuyên. Phát hiện P19-1 (đủ ĐK xin miễn ≠ cần), P19-2 (AV tăng cường trước căn bản), P19-3 (parser kì/kỳ, HK4, NFD). Hạn chế: chỉ 1 HK, chưa lịch học.</t>
+          <t>18/10/2026: Recommendation v1 (w19_recommendation/) — đề xuất đăng ký 1 HK (hk 1/2/3): ứng viên hợp lệ trên MỌI thế giới (du_dk_dang_ky TRUE, chưa tích lũy, mở HK, cần cho CTĐT; nhóm một nhánh), clingo tối ưu ≤20 TC (R-C01) + ưu tiên CHÍNH SÁCH (bắt buộc → mở khóa → nhóm → TC); UNKNOWN → cần xác minh; hình thức tốt nghiệp qua Eligibility; xin miễn (nộp đơn, QD-11); thay thế (R-M13). validate_recommendation 39/39 (tự soạn), bất biến kiểm lại độc lập 21 lần đề xuất, mọi tuần 5–19 ĐẠT. CẬP NHẬT: QD-13 RÚT LẠI sau khi đối chiếu PDF gốc — song hành theo đúng QĐ3266 Đ7 k5 (học trước/cùng lúc; đã học kể cả F, W không tính) → ràng buộc cứng. Trang 20 QĐ3266 (OCR trắng) đã chép tay từ PDF gốc. Phát hiện P19-1 (đủ ĐK xin miễn ≠ cần), P19-2 (AV tăng cường trước căn bản), P19-3 (parser kì/kỳ, HK4, NFD). Hạn chế: chỉ 1 HK, chưa lịch học.</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không có phần đọc tài liệu mới | Code: recommendation.py, recommendation.lp, prototype.answer_recommendation + parser de_xuat | Test: validate_recommendation 34/34 | Artifact: Tuan19_Recommendation.md | Lỗi/phát hiện: P19-1 đủ ĐK xin miễn ≠ cần; P19-2 ưu tiên TC chọn AV tăng cường trước căn bản; P19-3 parser học kỳ/ý định</t>
+          <t>Đọc: không có phần đọc tài liệu mới | Code: recommendation.py, recommendation.lp, prototype.answer_recommendation + parser de_xuat | Test: validate_recommendation 39/39 | Artifact: Tuan19_Recommendation.md | Lỗi/phát hiện: P19-1 đủ ĐK xin miễn ≠ cần; P19-2 ưu tiên TC chọn AV tăng cường trước căn bản; P19-3 parser học kỳ/ý định</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(w20): benchmark — chạy dev, đầu vào baseline, Q-Real pipeline, báo cáo Tuần 20
- run_cpa2 dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc
  nguyên — 3,14 không thuộc hạng nào; P20-2/3 parser ngoài phạm vi → tot_nghiep),
  OCR-Noise 100% sound, coverage 25% (P20-4: M2 từ chối thừa); test → Tuần 22
- review: id baseline mờ + đảo thứ tự (chống lộ đáp án); hash đóng băng mở rộng
  mọi trường chấm + hồ sơ gốc + CTĐT (tính trên đúng nội dung 312b7ff);
  phương án rỗng = từ chối; ghi claim parser; Q-Real ẩn danh link FB/mã lớp/MSSV
  có dấu cách, da_xoa không nhập lại
- baseline_dev/test.jsonl; qreal/ (0/400 — chờ câu hỏi thật)
- mọi tuần 5–20 ĐẠT

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1958,10 +1958,14 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>Hoàn thành một phần</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT; mọi tuần 5–20 ĐẠT. Test → Tuần 22.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2979,25 +2983,29 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
+          <t>☑</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>☐</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
+          <t>☑</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B9 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">

</xml_diff>

<commit_message>
fix(w5,w12): P20-1 hạng tốt nghiệp so hữu tỉ (R-Formal v1.10, QD-14); P20-2/3 parser
- hạng tốt nghiệp: bỏ mốc nguyên thang ×10 (3,14 / 3,57 / 2,45 không thuộc hạng
  nào); so hữu tỉ theo cận dưới; QD-14: QĐ3266 không làm tròn ĐTBCTL → giá trị
  giữa 3,59 và 3,60 thuộc Giỏi (catalog R-F06 + phụ lục sinh lại)
- parser: không mặc định tot_nghiep — câu không nhận ra → UNKNOWN "chưa hỗ trợ";
  "đăng ký <tên HP> <MÃ>" (khe chỉ là tên HP, không 'của/với/hủy/rút/gì/nào');
  luận văn → Eligibility; tốt nghiệp không dấu / "có thể" / "đăng kí … ko"
- ca hồi quy fail với luật/code cũ: rformal C42–C46, integration E10–E16
- G-Truth dev sau sửa 100% sound (_sau_P20; dev đã nhìn thấy — số chính thức
  là test ở Tuần 22); mọi tuần 5–20 ĐẠT

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT; mọi tuần 5–20 ĐẠT. Test → Tuần 22.</t>
+          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT.</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B9 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt</t>
+          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B9 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(w20): Q-Noise dev — chạy chính thức lần đầu, phát hiện P20-5
- dev 130 câu: Soundness 96,9%, Coverage 38,5%; V0 26/26, V1 bỏ dấu 84,6% sound,
  V2/V4 viết tắt coverage 0%, V3 gõ vội 20/26 đúng ý định
- P20-5 (an toàn, chưa sửa): "lam luan van tot nghiep" không dấu → parser hiểu tot_nghiep
  (4 unsound khi chấm chặt theo ý định, 2 theo gold thuần)
- Tuan20 §5c, Viec_ton_dong C13, README, CLAUDE.md Bài học, Excel H21/G21

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT.</t>
+          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep), chưa sửa.</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B9 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16</t>
+          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B10 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu (chưa sửa)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(w12): P20-5 parser chuẩn hoá cách gõ — bỏ dấu từ khoá, viết tắt theo ngữ cảnh, chặn câu hỏi mở
- chuan_hoa(): bỏ dấu CHỈ từ trong TU_KHOA (tránh thế→the, dự→du, nền→nen), mở viết tắt
  đk/tn theo ngữ cảnh, tl tn, lv/lvtn/tltn, hp, hk, đc, ko, e
- loại trừ không dấu + có dấu ở nhánh tốt nghiệp (luận văn, ĐTBCTL, lễ, thẻ, đồ án, thực tập …);
  HOI_MO chặn ý định có/không; đăng ký cần một mã HP + được/chưa/không, không "thì …"
- TLTN đọc từ câu đã chuẩn hoá; bỏ stub du_dk_dang_ky không đối số; học kỳ đề xuất đọc từ câu không dấu
- validate_integration E17–E28 (fail với code cũ); 2 lượt review đối kháng
- số sau sửa ra file _sau_P20-5 (dev đã thấy): Q-Noise dev 100% sound, 88,5% coverage

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep), chưa sửa.</t>
+          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep) → đã sửa (parser chuẩn hoá bỏ dấu từ khoá + viết tắt theo ngữ cảnh, E17–E28, 2 lượt review); sau sửa (dev đã thấy, file _sau_P20-5): Q-Noise 100% sound / 88,5% coverage, G-Truth không đổi.</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B10 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu (chưa sửa)</t>
+          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B10 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu → đã sửa, integration E17–E28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(w20): biểu mẫu thu câu hỏi + Q-Elicit 20 kịch bản (đóng băng), nhập CSV form + rút lại
- build_bieu_mau.py → qreal/bieu_mau.md: đồng ý theo NĐ 13/2023 (người thu/liên hệ để điền,
  mục đích, GitHub + dịch vụ AI, hạn xoá bản thô, mã rút lại + giới hạn), câu tự do hỏi TRƯỚC
  kịch bản, chọn bộ 1–4, không hỏi tên/MSSV/email/SĐT/ngày sinh
- qreal/kich_ban_q_elicit.json: 20 kịch bản viết tay, phủ 11 ý định, chống mớm lời,
  split theo kịch bản; đóng băng ở kich_ban_dong_bang.json
- nhap_qreal.py: nhận CSV form theo mã [..], chỉ dòng đồng ý, cảnh báo file/dòng bị bỏ,
  Q-Elicit ghi riêng qelicit.json (không tính vào Q-Real), nhieu_cau, --rut <mã> (bảng băm
  chỉ trong _tho/, câu trùng của người khác giữ lại)
- validate_benchmark B11a–h (nhập đầu–cuối trên dữ liệu giả, thư mục tạm); 2 lượt review
- Q-Real vẫn chưa đạt 0/400 — chờ phát form

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep) → đã sửa (parser chuẩn hoá bỏ dấu từ khoá + viết tắt theo ngữ cảnh, E17–E28, 2 lượt review); sau sửa (dev đã thấy, file _sau_P20-5): Q-Noise 100% sound / 88,5% coverage, G-Truth không đổi.</t>
+          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep) → đã sửa (parser chuẩn hoá bỏ dấu từ khoá + viết tắt theo ngữ cảnh, E17–E28, 2 lượt review); sau sửa (dev đã thấy, file _sau_P20-5): Q-Noise 100% sound / 88,5% coverage, G-Truth không đổi. | 19/10/2026: Google Form thu câu hỏi (đồng ý NĐ 13/2023, mã rút lại, câu tự do trước kịch bản) + Q-Elicit 20 kịch bản đóng băng (báo riêng, không tính); Q-Real vẫn chưa đạt 0/400 — chờ Loi phát form.</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B10 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu → đã sửa, integration E17–E28</t>
+          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B11 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu → đã sửa, integration E17–E28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(w15): P20-4 mất ĐTBCHK — giữ từ chối, hỏi đúng một số ĐTBCHK in, nhận khai báo số in
- M2 (bảng sạch mất ĐTBCHK) không phân biệt được với F1 (đọc nhầm F→D + mất ĐTBCHK) →
  vẫn không tin điểm học kỳ (P17-2)
- bc["can_hoi"]: một mục dtbchk:<học kỳ> thay cho 5–7 HP; khai_bao["dtbchk_khai_bao"]
  khôi phục kiểm chéo (khớp → tin, lệch → vẫn không tin); số OCR đọc được thắng khai báo
- khai báo chỉ nhận số hữu hạn trong [0,4] (review: NaN làm học kỳ được tin), "3,08",
  tên học kỳ chuẩn hoá, lỗi khai báo báo ở bc["khai_bao_loi"]; học kỳ lệch tổng TC không dùng
- validate_ocr F5–F11; run_cpa2 đường OCR trả can_hoi
- OCR-Noise dev _sau_P20-4: số không đổi (0 unsound, M2 0% coverage); phương án B (số
  tích lũy) để kế hoạch riêng (C14)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep) → đã sửa (parser chuẩn hoá bỏ dấu từ khoá + viết tắt theo ngữ cảnh, E17–E28, 2 lượt review); sau sửa (dev đã thấy, file _sau_P20-5): Q-Noise 100% sound / 88,5% coverage, G-Truth không đổi. | 19/10/2026: Google Form thu câu hỏi (đồng ý NĐ 13/2023, mã rút lại, câu tự do trước kịch bản) + Q-Elicit 20 kịch bản đóng băng (báo riêng, không tính); Q-Real vẫn chưa đạt 0/400 — chờ Loi phát form.</t>
+          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep) → đã sửa (parser chuẩn hoá bỏ dấu từ khoá + viết tắt theo ngữ cảnh, E17–E28, 2 lượt review); sau sửa (dev đã thấy, file _sau_P20-5): Q-Noise 100% sound / 88,5% coverage, G-Truth không đổi. | 19/10/2026: Google Form thu câu hỏi (đồng ý NĐ 13/2023, mã rút lại, câu tự do trước kịch bản) + Q-Elicit 20 kịch bản đóng băng (báo riêng, không tính); Q-Real vẫn chưa đạt 0/400 — chờ Loi phát form. | P20-4 (A): mất ĐTBCHK vẫn không tin điểm (M2 ≡ F1), hỏi 1 số ĐTBCHK in thay 5–7 HP, nhận khai báo số in (validate_ocr F5–F11); OCR-Noise dev không đổi (M2 0% coverage), mô phỏng trả lời → 5/5 TRUE. Phương án B (số tích lũy) lập kế hoạch riêng.</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B11 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu → đã sửa, integration E17–E28</t>
+          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B11 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu → đã sửa, integration E17–E28 | P20-4: w15 F5–F11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(w15,w17): C14 kiểm chéo OCR bằng số tích lũy in sau mỗi học kỳ + bịt lỗ GDTC F→D
- Đọc "Tổng Số Tín Chỉ Tích Lũy" + "Điểm T.Bình chung tích lũy" mỗi học kỳ.
- Luôn kiểm TC tích lũy khi đọc được: GDTC thật F đọc nhất quán thành D
  (ĐTBCHK không tính GDTC, R-B08) từng cho TRUE sai; dòng GDTC chỉ được tin
  qua phép thử lật giả thuyết (bao mọi độ chùng).
- Cứu học kỳ mất ĐTBCHK khi học kỳ trước đã tin, TC khớp chính xác, ĐTBCTL
  khớp và đủ độ phân giải; GDQP vẫn không chắc; có dòng miễn mà chưa biết
  quy ước (MIEN_TRONG_TC_TICH_LUY) thì không cứu. Mã GDTC thật TC025–027.
- render_transcript: CC004 vào TC tích lũy mọi học kỳ sau; w17 dau_vao sinh
  số tích lũy độc lập (oracle).
- validate_ocr G0–G15 + G11 ảnh; OCR-Noise dev M2 0/5 → 4/5, Sound 100%.
- Báo cáo Tuần 20 §5g, Viec_ton_dong (C14 đóng, A18), Bài học, Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014n9qXppK2zJNGmYoQK5HFw
</commit_message>
<xml_diff>
--- a/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
+++ b/Ke_hoach_nghien_cuu_CPA2_24_tuan.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep) → đã sửa (parser chuẩn hoá bỏ dấu từ khoá + viết tắt theo ngữ cảnh, E17–E28, 2 lượt review); sau sửa (dev đã thấy, file _sau_P20-5): Q-Noise 100% sound / 88,5% coverage, G-Truth không đổi. | 19/10/2026: Google Form thu câu hỏi (đồng ý NĐ 13/2023, mã rút lại, câu tự do trước kịch bản) + Q-Elicit 20 kịch bản đóng băng (báo riêng, không tính); Q-Real vẫn chưa đạt 0/400 — chờ Loi phát form. | P20-4 (A): mất ĐTBCHK vẫn không tin điểm (M2 ≡ F1), hỏi 1 số ĐTBCHK in thay 5–7 HP, nhận khai báo số in (validate_ocr F5–F11); OCR-Noise dev không đổi (M2 0% coverage), mô phỏng trả lời → 5/5 TRUE. Phương án B (số tích lũy) lập kế hoạch riêng. | C12: ý định xếp loại tốt nghiệp (QD-15 đúng hạng; E29–E37); review phát hiện C15 — KB không hạ bậc (tc_diem_f không sinh, Đ34 k2 b chưa hình thức hoá) → prototype trả UNKNOWN với hạng gốc XS/G; sửa R-Formal lập kế hoạch riêng (ảnh hưởng gold HG). | C15: R-Formal v1.11 — hạ bậc Đ34 k2 a+b (HP điểm cuối F chắc chắn; tc_diem_f, kỷ luật cấp Trường là khai báo; chưa khai báo → mở nhánh), R-F07b; errata G-Truth HG-02/03/04/08; dev chính thức 57/58 (HG-03 từ chối thừa), theo errata 58/58. A17 hỏi HP điều kiện.</t>
+          <t>18/10/2026: w20_benchmark/ — G-Truth v1 115 ca (114 chấm) + OCR-Noise v1 40 ca, gold viết tay + nguồn + oracle độc lập (41 tiền đề), loai_gold quy_che/thiet_ke, soát độc lập (không chạy hệ thống) rồi ĐÓNG BĂNG 312b7ff trước lần chạy đầu; không trùng w17; dev/test. Đầu vào baseline trung lập (baseline_dev/test.jsonl). Q-Real: pipeline nhập/ẩn danh xong, CHƯA ĐẠT 0/400 (chờ câu hỏi thật). Chạy dev: G-Truth Soundness 89,7% (6 unsound: P20-1 hạng tốt nghiệp mốc nguyên, P20-2/3 parser), OCR-Noise 100% sound, coverage 25% (M2 từ chối thừa). validate_benchmark ĐẠT. SỬA P20-1 (R-Formal v1.10: hạng so hữu tỉ theo cận dưới, QD-14 không làm tròn ĐTBCTL), P20-2 (parser không mặc định tot_nghiep → UNKNOWN 'chưa hỗ trợ'), P20-3 (đăng ký có tên HP chen giữa) — ca hồi quy fail với luật cũ; G-Truth dev sau sửa 100% sound (dev đã nhìn thấy; số chính thức = test, Tuần 22). Còn: Q-Real 0/400, P20-4. Mọi tuần 5–20 ĐẠT. | Q-Noise v1 (TỔNG HỢP, không thay Q-Real): 240 câu = 48 câu G-Truth × 5 kiểu gõ (gốc/bỏ dấu/viết tắt/gõ vội/bỏ dấu+viết tắt), gold kế thừa + ý định gán tay, đóng băng 5d8601c; dev: Sound 96,9%, Coverage 38,5% (V2/V4 0%), phát hiện P20-5 (4 unsound: luan van không dấu → tot_nghiep) → đã sửa (parser chuẩn hoá bỏ dấu từ khoá + viết tắt theo ngữ cảnh, E17–E28, 2 lượt review); sau sửa (dev đã thấy, file _sau_P20-5): Q-Noise 100% sound / 88,5% coverage, G-Truth không đổi. | 19/10/2026: Google Form thu câu hỏi (đồng ý NĐ 13/2023, mã rút lại, câu tự do trước kịch bản) + Q-Elicit 20 kịch bản đóng băng (báo riêng, không tính); Q-Real vẫn chưa đạt 0/400 — chờ Loi phát form. | P20-4 (A): mất ĐTBCHK vẫn không tin điểm (M2 ≡ F1), hỏi 1 số ĐTBCHK in thay 5–7 HP, nhận khai báo số in (validate_ocr F5–F11); OCR-Noise dev không đổi (M2 0% coverage), mô phỏng trả lời → 5/5 TRUE. Phương án B (số tích lũy) lập kế hoạch riêng. | C12: ý định xếp loại tốt nghiệp (QD-15 đúng hạng; E29–E37); review phát hiện C15 — KB không hạ bậc (tc_diem_f không sinh, Đ34 k2 b chưa hình thức hoá) → prototype trả UNKNOWN với hạng gốc XS/G; sửa R-Formal lập kế hoạch riêng (ảnh hưởng gold HG). | C15: R-Formal v1.11 — hạ bậc Đ34 k2 a+b (HP điểm cuối F chắc chắn; tc_diem_f, kỷ luật cấp Trường là khai báo; chưa khai báo → mở nhánh), R-F07b; errata G-Truth HG-02/03/04/08; dev chính thức 57/58 (HG-03 từ chối thừa), theo errata 58/58. A17 hỏi HP điều kiện. | C14: kiểm chéo bằng TC tích lũy + ĐTBCTL in sau mỗi học kỳ — cứu học kỳ mất ĐTBCHK khi đủ độ phân giải, luôn kiểm TC tích lũy (bịt lỗ GDTC F→D cho TRUE sai); OCR-Noise dev M2 0/5 → 4/5, Sound 100%. A18: kiểm trên ảnh bảng điểm thật (Windows).</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B11 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu → đã sửa, integration E17–E28 | P20-4: w15 F5–F11 | C12: integration E29–E37, QD-15 | C15: rformal C47–C53, graduation D1–D4, student_facts L5, integration E42</t>
+          <t>Đọc: không | Code: build_benchmark.py, validate_benchmark.py, run_cpa2.py, baseline.py, nhap_qreal.py | Test: validate_benchmark B1–B11 ĐẠT | Artifact: Tuan20_Benchmark.md, gtruth.json, ocr_noise.json | Lỗi/phát hiện: P20-1 hạng TN mốc nguyên; P20-2 ngoài phạm vi → tot_nghiep; P20-3 đăng ký niên luận; P20-4 OCR M2 từ chối thừa; Q-Real 0/400 chưa đạt | Sửa: P20-1 (v1.10, QD-14), P20-2, P20-3 — rformal C42–C46, integration E10–E16 | Q-Noise: P20-5 parser không dấu → đã sửa, integration E17–E28 | P20-4: w15 F5–F11 | C12: integration E29–E37, QD-15 | C15: rformal C47–C53, graduation D1–D4, student_facts L5, integration E42 | C14: w15 G0–G15 + G11 ảnh (G9/G12/G13/G15 fail trước sửa)</t>
         </is>
       </c>
     </row>

</xml_diff>